<commit_message>
Update files (new languages)
</commit_message>
<xml_diff>
--- a/OpenSesame-local/Language_localiser.xlsx
+++ b/OpenSesame-local/Language_localiser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdabb12e9f34f4c5/10_Paper/105_MIA/10_BAS_Collab/MBRT/OpenSesame-local/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{439F560A-EC9A-4A85-BCCA-B610A865D2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAB2DAFC-6248-4BD5-A876-C8706B198FD8}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{439F560A-EC9A-4A85-BCCA-B610A865D2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1320B2DF-685A-4026-ADD2-4EFD69591932}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36299" yWindow="1250" windowWidth="26083" windowHeight="13829" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -96,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>language</t>
   </si>
@@ -114,6 +117,18 @@
   </si>
   <si>
     <t>DE</t>
+  </si>
+  <si>
+    <t>Spanish</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>French</t>
+  </si>
+  <si>
+    <t>FR</t>
   </si>
 </sst>
 </file>
@@ -215,9 +230,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -255,7 +270,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -361,7 +376,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -503,7 +518,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -511,10 +526,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="20.7109375" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.75" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="1"/>
+    <col min="1" max="1" width="20.75" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -539,6 +554,22 @@
       </c>
       <c r="B3" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -668,18 +699,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -699,14 +730,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -719,4 +742,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>